<commit_message>
feat(questions): allow nullable question and option content by TOEIC part
</commit_message>
<xml_diff>
--- a/apps/backend/test/fixtures/questions_valid_small.xlsx
+++ b/apps/backend/test/fixtures/questions_valid_small.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="38">
   <si>
     <t>Part</t>
   </si>
@@ -116,6 +116,15 @@
   </si>
   <si>
     <t>vocabulary</t>
+  </si>
+  <si>
+    <t>Audio explanation for Part 1</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Audio explanation for Part 2</t>
   </si>
 </sst>
 </file>
@@ -492,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -636,8 +645,102 @@
         <v>25</v>
       </c>
     </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" t="s">
+        <v>25</v>
+      </c>
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M5" t="s">
+        <v>25</v>
+      </c>
+      <c r="N5" t="s">
+        <v>25</v>
+      </c>
+      <c r="O5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>